<commit_message>
Update formatting of dates in Excel data spreadsheets
</commit_message>
<xml_diff>
--- a/data/cyano_atx_24.xlsx
+++ b/data/cyano_atx_24.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jld/Documents/Github/River_HAB_Modeling/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{516D896E-94C5-6040-90A9-0D5214DC8149}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0916428D-C709-DE44-AC02-AC5130F9B77E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="800" yWindow="760" windowWidth="27700" windowHeight="18040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -690,8 +690,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.000"/>
+    <numFmt numFmtId="166" formatCode="yyyy\-mm\-dd;@"/>
+    <numFmt numFmtId="167" formatCode="[$-409]mmmm\ d\,\ yyyy;@"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -751,7 +753,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -761,6 +763,12 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1068,6 +1076,7 @@
   <dimension ref="A1:U120"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
+    <col min="3" max="3" width="8.83203125" style="6"/>
     <col min="21" max="21" width="9.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1078,7 +1087,7 @@
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
@@ -1128,7 +1137,7 @@
       <c r="B2" t="s">
         <v>134</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="8" t="s">
         <v>179</v>
       </c>
       <c r="D2" t="s">
@@ -1176,7 +1185,7 @@
       <c r="B3" t="s">
         <v>135</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="8" t="s">
         <v>179</v>
       </c>
       <c r="D3" t="s">
@@ -1223,7 +1232,7 @@
       <c r="B4" t="s">
         <v>136</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="8" t="s">
         <v>179</v>
       </c>
       <c r="D4" t="s">
@@ -1270,7 +1279,7 @@
       <c r="B5" t="s">
         <v>137</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="8" t="s">
         <v>180</v>
       </c>
       <c r="D5" t="s">
@@ -1317,7 +1326,7 @@
       <c r="B6" t="s">
         <v>138</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="8" t="s">
         <v>180</v>
       </c>
       <c r="D6" t="s">
@@ -1364,7 +1373,7 @@
       <c r="B7" t="s">
         <v>139</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="8" t="s">
         <v>180</v>
       </c>
       <c r="D7" t="s">
@@ -1411,7 +1420,7 @@
       <c r="B8" t="s">
         <v>140</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="8" t="s">
         <v>180</v>
       </c>
       <c r="D8" t="s">
@@ -1458,7 +1467,7 @@
       <c r="B9" t="s">
         <v>141</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="8" t="s">
         <v>181</v>
       </c>
       <c r="D9" t="s">
@@ -1505,7 +1514,7 @@
       <c r="B10" t="s">
         <v>142</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="8" t="s">
         <v>181</v>
       </c>
       <c r="D10" t="s">
@@ -1552,7 +1561,7 @@
       <c r="B11" t="s">
         <v>143</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="8" t="s">
         <v>182</v>
       </c>
       <c r="D11" t="s">
@@ -1599,7 +1608,7 @@
       <c r="B12" t="s">
         <v>144</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" s="8" t="s">
         <v>182</v>
       </c>
       <c r="D12" t="s">
@@ -1646,7 +1655,7 @@
       <c r="B13" t="s">
         <v>145</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" s="8" t="s">
         <v>182</v>
       </c>
       <c r="D13" t="s">
@@ -1693,7 +1702,7 @@
       <c r="B14" t="s">
         <v>146</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C14" s="8" t="s">
         <v>182</v>
       </c>
       <c r="D14" t="s">
@@ -1740,7 +1749,7 @@
       <c r="B15" t="s">
         <v>147</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C15" s="8" t="s">
         <v>183</v>
       </c>
       <c r="D15" t="s">
@@ -1787,7 +1796,7 @@
       <c r="B16" t="s">
         <v>148</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C16" s="8" t="s">
         <v>183</v>
       </c>
       <c r="D16" t="s">
@@ -1834,7 +1843,7 @@
       <c r="B17" t="s">
         <v>149</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C17" s="8" t="s">
         <v>184</v>
       </c>
       <c r="D17" t="s">
@@ -1881,7 +1890,7 @@
       <c r="B18" t="s">
         <v>149</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C18" s="8" t="s">
         <v>185</v>
       </c>
       <c r="D18" t="s">
@@ -1928,7 +1937,7 @@
       <c r="B19" t="s">
         <v>149</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C19" s="8" t="s">
         <v>185</v>
       </c>
       <c r="D19" t="s">
@@ -1975,7 +1984,7 @@
       <c r="B20" t="s">
         <v>150</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C20" s="8" t="s">
         <v>185</v>
       </c>
       <c r="D20" t="s">
@@ -2022,7 +2031,7 @@
       <c r="B21" t="s">
         <v>151</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C21" s="8" t="s">
         <v>185</v>
       </c>
       <c r="D21" t="s">
@@ -2069,7 +2078,7 @@
       <c r="B22" t="s">
         <v>152</v>
       </c>
-      <c r="C22" t="s">
+      <c r="C22" s="8" t="s">
         <v>185</v>
       </c>
       <c r="D22" t="s">
@@ -2116,7 +2125,7 @@
       <c r="B23" t="s">
         <v>150</v>
       </c>
-      <c r="C23" t="s">
+      <c r="C23" s="8" t="s">
         <v>185</v>
       </c>
       <c r="D23" t="s">
@@ -2163,7 +2172,7 @@
       <c r="B24" t="s">
         <v>151</v>
       </c>
-      <c r="C24" t="s">
+      <c r="C24" s="8" t="s">
         <v>185</v>
       </c>
       <c r="D24" t="s">
@@ -2210,7 +2219,7 @@
       <c r="B25" t="s">
         <v>152</v>
       </c>
-      <c r="C25" t="s">
+      <c r="C25" s="8" t="s">
         <v>185</v>
       </c>
       <c r="D25" t="s">
@@ -2257,7 +2266,7 @@
       <c r="B26" t="s">
         <v>153</v>
       </c>
-      <c r="C26" t="s">
+      <c r="C26" s="7" t="s">
         <v>186</v>
       </c>
       <c r="D26" t="s">
@@ -2304,7 +2313,7 @@
       <c r="B27" t="s">
         <v>154</v>
       </c>
-      <c r="C27" t="s">
+      <c r="C27" s="7" t="s">
         <v>185</v>
       </c>
       <c r="D27" t="s">
@@ -2351,7 +2360,7 @@
       <c r="B28" t="s">
         <v>154</v>
       </c>
-      <c r="C28" t="s">
+      <c r="C28" s="7" t="s">
         <v>185</v>
       </c>
       <c r="D28" t="s">
@@ -2398,7 +2407,7 @@
       <c r="B29" t="s">
         <v>155</v>
       </c>
-      <c r="C29" t="s">
+      <c r="C29" s="7" t="s">
         <v>185</v>
       </c>
       <c r="D29" t="s">
@@ -2445,7 +2454,7 @@
       <c r="B30" t="s">
         <v>155</v>
       </c>
-      <c r="C30" t="s">
+      <c r="C30" s="7" t="s">
         <v>185</v>
       </c>
       <c r="D30" t="s">
@@ -2492,7 +2501,7 @@
       <c r="B31" t="s">
         <v>149</v>
       </c>
-      <c r="C31" t="s">
+      <c r="C31" s="7" t="s">
         <v>187</v>
       </c>
       <c r="D31" t="s">
@@ -2539,7 +2548,7 @@
       <c r="B32" t="s">
         <v>149</v>
       </c>
-      <c r="C32" t="s">
+      <c r="C32" s="7" t="s">
         <v>187</v>
       </c>
       <c r="D32" t="s">
@@ -2586,7 +2595,7 @@
       <c r="B33" t="s">
         <v>156</v>
       </c>
-      <c r="C33" t="s">
+      <c r="C33" s="7" t="s">
         <v>187</v>
       </c>
       <c r="D33" t="s">
@@ -2633,7 +2642,7 @@
       <c r="B34" t="s">
         <v>157</v>
       </c>
-      <c r="C34" t="s">
+      <c r="C34" s="7" t="s">
         <v>187</v>
       </c>
       <c r="D34" t="s">
@@ -2680,7 +2689,7 @@
       <c r="B35" t="s">
         <v>149</v>
       </c>
-      <c r="C35" t="s">
+      <c r="C35" s="7" t="s">
         <v>187</v>
       </c>
       <c r="D35" t="s">
@@ -2727,7 +2736,7 @@
       <c r="B36" t="s">
         <v>150</v>
       </c>
-      <c r="C36" t="s">
+      <c r="C36" s="7" t="s">
         <v>187</v>
       </c>
       <c r="D36" t="s">
@@ -2774,7 +2783,7 @@
       <c r="B37" t="s">
         <v>150</v>
       </c>
-      <c r="C37" t="s">
+      <c r="C37" s="7" t="s">
         <v>187</v>
       </c>
       <c r="D37" t="s">
@@ -2821,7 +2830,7 @@
       <c r="B38" t="s">
         <v>154</v>
       </c>
-      <c r="C38" t="s">
+      <c r="C38" s="7" t="s">
         <v>187</v>
       </c>
       <c r="D38" t="s">
@@ -2868,7 +2877,7 @@
       <c r="B39" t="s">
         <v>154</v>
       </c>
-      <c r="C39" t="s">
+      <c r="C39" s="7" t="s">
         <v>187</v>
       </c>
       <c r="D39" t="s">
@@ -2915,7 +2924,7 @@
       <c r="B40" t="s">
         <v>155</v>
       </c>
-      <c r="C40" t="s">
+      <c r="C40" s="7" t="s">
         <v>187</v>
       </c>
       <c r="D40" t="s">
@@ -2962,7 +2971,7 @@
       <c r="B41" t="s">
         <v>155</v>
       </c>
-      <c r="C41" t="s">
+      <c r="C41" s="7" t="s">
         <v>187</v>
       </c>
       <c r="D41" t="s">
@@ -3009,7 +3018,7 @@
       <c r="B42" t="s">
         <v>149</v>
       </c>
-      <c r="C42" t="s">
+      <c r="C42" s="7" t="s">
         <v>188</v>
       </c>
       <c r="D42" t="s">
@@ -3056,7 +3065,7 @@
       <c r="B43" t="s">
         <v>158</v>
       </c>
-      <c r="C43" t="s">
+      <c r="C43" s="7" t="s">
         <v>188</v>
       </c>
       <c r="D43" t="s">
@@ -3103,7 +3112,7 @@
       <c r="B44" t="s">
         <v>149</v>
       </c>
-      <c r="C44" t="s">
+      <c r="C44" s="7" t="s">
         <v>188</v>
       </c>
       <c r="D44" t="s">
@@ -3150,7 +3159,7 @@
       <c r="B45" t="s">
         <v>158</v>
       </c>
-      <c r="C45" t="s">
+      <c r="C45" s="7" t="s">
         <v>188</v>
       </c>
       <c r="D45" t="s">
@@ -3197,7 +3206,7 @@
       <c r="B46" t="s">
         <v>159</v>
       </c>
-      <c r="C46" t="s">
+      <c r="C46" s="7" t="s">
         <v>186</v>
       </c>
       <c r="D46" t="s">
@@ -3244,7 +3253,7 @@
       <c r="B47" t="s">
         <v>150</v>
       </c>
-      <c r="C47" t="s">
+      <c r="C47" s="7" t="s">
         <v>188</v>
       </c>
       <c r="D47" t="s">
@@ -3291,7 +3300,7 @@
       <c r="B48" t="s">
         <v>150</v>
       </c>
-      <c r="C48" t="s">
+      <c r="C48" s="7" t="s">
         <v>188</v>
       </c>
       <c r="D48" t="s">
@@ -3338,7 +3347,7 @@
       <c r="B49" t="s">
         <v>154</v>
       </c>
-      <c r="C49" t="s">
+      <c r="C49" s="7" t="s">
         <v>188</v>
       </c>
       <c r="D49" t="s">
@@ -3385,7 +3394,7 @@
       <c r="B50" t="s">
         <v>154</v>
       </c>
-      <c r="C50" t="s">
+      <c r="C50" s="7" t="s">
         <v>188</v>
       </c>
       <c r="D50" t="s">
@@ -3432,7 +3441,7 @@
       <c r="B51" t="s">
         <v>155</v>
       </c>
-      <c r="C51" t="s">
+      <c r="C51" s="7" t="s">
         <v>188</v>
       </c>
       <c r="D51" t="s">
@@ -3479,7 +3488,7 @@
       <c r="B52" t="s">
         <v>160</v>
       </c>
-      <c r="C52" t="s">
+      <c r="C52" s="7" t="s">
         <v>188</v>
       </c>
       <c r="D52" t="s">
@@ -3526,7 +3535,7 @@
       <c r="B53" t="s">
         <v>161</v>
       </c>
-      <c r="C53" t="s">
+      <c r="C53" s="7" t="s">
         <v>188</v>
       </c>
       <c r="D53" t="s">
@@ -3573,7 +3582,7 @@
       <c r="B54" t="s">
         <v>155</v>
       </c>
-      <c r="C54" t="s">
+      <c r="C54" s="7" t="s">
         <v>188</v>
       </c>
       <c r="D54" t="s">
@@ -3620,7 +3629,7 @@
       <c r="B55" t="s">
         <v>160</v>
       </c>
-      <c r="C55" t="s">
+      <c r="C55" s="7" t="s">
         <v>188</v>
       </c>
       <c r="D55" t="s">
@@ -3667,7 +3676,7 @@
       <c r="B56" t="s">
         <v>161</v>
       </c>
-      <c r="C56" t="s">
+      <c r="C56" s="7" t="s">
         <v>188</v>
       </c>
       <c r="D56" t="s">
@@ -3714,7 +3723,7 @@
       <c r="B57" t="s">
         <v>148</v>
       </c>
-      <c r="C57" t="s">
+      <c r="C57" s="7" t="s">
         <v>189</v>
       </c>
       <c r="D57" t="s">
@@ -3761,7 +3770,7 @@
       <c r="B58" t="s">
         <v>136</v>
       </c>
-      <c r="C58" t="s">
+      <c r="C58" s="7" t="s">
         <v>189</v>
       </c>
       <c r="D58" t="s">
@@ -3808,7 +3817,7 @@
       <c r="B59" t="s">
         <v>146</v>
       </c>
-      <c r="C59" t="s">
+      <c r="C59" s="7" t="s">
         <v>189</v>
       </c>
       <c r="D59" t="s">
@@ -3855,7 +3864,7 @@
       <c r="B60" t="s">
         <v>162</v>
       </c>
-      <c r="C60" t="s">
+      <c r="C60" s="7" t="s">
         <v>189</v>
       </c>
       <c r="D60" t="s">
@@ -3902,7 +3911,7 @@
       <c r="B61" t="s">
         <v>145</v>
       </c>
-      <c r="C61" t="s">
+      <c r="C61" s="7" t="s">
         <v>190</v>
       </c>
       <c r="D61" t="s">
@@ -3949,7 +3958,7 @@
       <c r="B62" t="s">
         <v>163</v>
       </c>
-      <c r="C62" t="s">
+      <c r="C62" s="7" t="s">
         <v>190</v>
       </c>
       <c r="D62" t="s">
@@ -3996,7 +4005,7 @@
       <c r="B63" t="s">
         <v>147</v>
       </c>
-      <c r="C63" t="s">
+      <c r="C63" s="7" t="s">
         <v>190</v>
       </c>
       <c r="D63" t="s">
@@ -4043,7 +4052,7 @@
       <c r="B64" t="s">
         <v>142</v>
       </c>
-      <c r="C64" t="s">
+      <c r="C64" s="7" t="s">
         <v>191</v>
       </c>
       <c r="D64" t="s">
@@ -4090,7 +4099,7 @@
       <c r="B65" t="s">
         <v>134</v>
       </c>
-      <c r="C65" t="s">
+      <c r="C65" s="7" t="s">
         <v>192</v>
       </c>
       <c r="D65" t="s">
@@ -4137,7 +4146,7 @@
       <c r="B66" t="s">
         <v>140</v>
       </c>
-      <c r="C66" t="s">
+      <c r="C66" s="7" t="s">
         <v>193</v>
       </c>
       <c r="D66" t="s">
@@ -4184,7 +4193,7 @@
       <c r="B67" t="s">
         <v>164</v>
       </c>
-      <c r="C67" t="s">
+      <c r="C67" s="7" t="s">
         <v>193</v>
       </c>
       <c r="D67" t="s">
@@ -4231,7 +4240,7 @@
       <c r="B68" t="s">
         <v>144</v>
       </c>
-      <c r="C68" t="s">
+      <c r="C68" s="7" t="s">
         <v>194</v>
       </c>
       <c r="D68" t="s">
@@ -4278,7 +4287,7 @@
       <c r="B69" t="s">
         <v>147</v>
       </c>
-      <c r="C69" t="s">
+      <c r="C69" s="7" t="s">
         <v>195</v>
       </c>
       <c r="D69" t="s">
@@ -4325,7 +4334,7 @@
       <c r="B70" t="s">
         <v>145</v>
       </c>
-      <c r="C70" t="s">
+      <c r="C70" s="7" t="s">
         <v>195</v>
       </c>
       <c r="D70" t="s">
@@ -4372,7 +4381,7 @@
       <c r="B71" t="s">
         <v>165</v>
       </c>
-      <c r="C71" t="s">
+      <c r="C71" s="7" t="s">
         <v>186</v>
       </c>
       <c r="D71" t="s">
@@ -4419,7 +4428,7 @@
       <c r="B72" t="s">
         <v>149</v>
       </c>
-      <c r="C72" t="s">
+      <c r="C72" s="7" t="s">
         <v>196</v>
       </c>
       <c r="D72" t="s">
@@ -4466,7 +4475,7 @@
       <c r="B73" t="s">
         <v>149</v>
       </c>
-      <c r="C73" t="s">
+      <c r="C73" s="7" t="s">
         <v>196</v>
       </c>
       <c r="D73" t="s">
@@ -4513,7 +4522,7 @@
       <c r="B74" t="s">
         <v>150</v>
       </c>
-      <c r="C74" t="s">
+      <c r="C74" s="7" t="s">
         <v>196</v>
       </c>
       <c r="D74" t="s">
@@ -4560,7 +4569,7 @@
       <c r="B75" t="s">
         <v>150</v>
       </c>
-      <c r="C75" t="s">
+      <c r="C75" s="7" t="s">
         <v>196</v>
       </c>
       <c r="D75" t="s">
@@ -4607,7 +4616,7 @@
       <c r="B76" t="s">
         <v>154</v>
       </c>
-      <c r="C76" t="s">
+      <c r="C76" s="7" t="s">
         <v>196</v>
       </c>
       <c r="D76" t="s">
@@ -4654,7 +4663,7 @@
       <c r="B77" t="s">
         <v>166</v>
       </c>
-      <c r="C77" t="s">
+      <c r="C77" s="7" t="s">
         <v>196</v>
       </c>
       <c r="D77" t="s">
@@ -4701,7 +4710,7 @@
       <c r="B78" t="s">
         <v>167</v>
       </c>
-      <c r="C78" t="s">
+      <c r="C78" s="7" t="s">
         <v>196</v>
       </c>
       <c r="D78" t="s">
@@ -4748,7 +4757,7 @@
       <c r="B79" t="s">
         <v>168</v>
       </c>
-      <c r="C79" t="s">
+      <c r="C79" s="7" t="s">
         <v>196</v>
       </c>
       <c r="D79" t="s">
@@ -4795,7 +4804,7 @@
       <c r="B80" t="s">
         <v>155</v>
       </c>
-      <c r="C80" t="s">
+      <c r="C80" s="7" t="s">
         <v>196</v>
       </c>
       <c r="D80" t="s">
@@ -4842,7 +4851,7 @@
       <c r="B81" t="s">
         <v>155</v>
       </c>
-      <c r="C81" t="s">
+      <c r="C81" s="7" t="s">
         <v>196</v>
       </c>
       <c r="D81" t="s">
@@ -4889,7 +4898,7 @@
       <c r="B82" t="s">
         <v>139</v>
       </c>
-      <c r="C82" t="s">
+      <c r="C82" s="7" t="s">
         <v>197</v>
       </c>
       <c r="D82" t="s">
@@ -4936,7 +4945,7 @@
       <c r="B83" t="s">
         <v>138</v>
       </c>
-      <c r="C83" t="s">
+      <c r="C83" s="7" t="s">
         <v>197</v>
       </c>
       <c r="D83" t="s">
@@ -4983,7 +4992,7 @@
       <c r="B84" t="s">
         <v>136</v>
       </c>
-      <c r="C84" t="s">
+      <c r="C84" s="7" t="s">
         <v>197</v>
       </c>
       <c r="D84" t="s">
@@ -5030,7 +5039,7 @@
       <c r="B85" t="s">
         <v>143</v>
       </c>
-      <c r="C85" t="s">
+      <c r="C85" s="7" t="s">
         <v>198</v>
       </c>
       <c r="D85" t="s">
@@ -5077,7 +5086,7 @@
       <c r="B86" t="s">
         <v>145</v>
       </c>
-      <c r="C86" t="s">
+      <c r="C86" s="7" t="s">
         <v>198</v>
       </c>
       <c r="D86" t="s">
@@ -5124,7 +5133,7 @@
       <c r="B87" t="s">
         <v>148</v>
       </c>
-      <c r="C87" t="s">
+      <c r="C87" s="7" t="s">
         <v>199</v>
       </c>
       <c r="D87" t="s">
@@ -5171,7 +5180,7 @@
       <c r="B88" t="s">
         <v>141</v>
       </c>
-      <c r="C88" t="s">
+      <c r="C88" s="7" t="s">
         <v>199</v>
       </c>
       <c r="D88" t="s">
@@ -5218,7 +5227,7 @@
       <c r="B89" t="s">
         <v>149</v>
       </c>
-      <c r="C89" t="s">
+      <c r="C89" s="7" t="s">
         <v>200</v>
       </c>
       <c r="D89" t="s">
@@ -5265,7 +5274,7 @@
       <c r="B90" t="s">
         <v>150</v>
       </c>
-      <c r="C90" t="s">
+      <c r="C90" s="7" t="s">
         <v>200</v>
       </c>
       <c r="D90" t="s">
@@ -5312,7 +5321,7 @@
       <c r="B91" t="s">
         <v>151</v>
       </c>
-      <c r="C91" t="s">
+      <c r="C91" s="7" t="s">
         <v>200</v>
       </c>
       <c r="D91" t="s">
@@ -5359,7 +5368,7 @@
       <c r="B92" t="s">
         <v>169</v>
       </c>
-      <c r="C92" t="s">
+      <c r="C92" s="7" t="s">
         <v>200</v>
       </c>
       <c r="D92" t="s">
@@ -5406,7 +5415,7 @@
       <c r="B93" t="s">
         <v>154</v>
       </c>
-      <c r="C93" t="s">
+      <c r="C93" s="7" t="s">
         <v>200</v>
       </c>
       <c r="D93" t="s">
@@ -5453,7 +5462,7 @@
       <c r="B94" t="s">
         <v>155</v>
       </c>
-      <c r="C94" t="s">
+      <c r="C94" s="7" t="s">
         <v>200</v>
       </c>
       <c r="D94" t="s">
@@ -5500,7 +5509,7 @@
       <c r="B95" t="s">
         <v>149</v>
       </c>
-      <c r="C95" t="s">
+      <c r="C95" s="7" t="s">
         <v>201</v>
       </c>
       <c r="D95" t="s">
@@ -5547,7 +5556,7 @@
       <c r="B96" t="s">
         <v>156</v>
       </c>
-      <c r="C96" t="s">
+      <c r="C96" s="7" t="s">
         <v>201</v>
       </c>
       <c r="D96" t="s">
@@ -5594,7 +5603,7 @@
       <c r="B97" t="s">
         <v>157</v>
       </c>
-      <c r="C97" t="s">
+      <c r="C97" s="7" t="s">
         <v>201</v>
       </c>
       <c r="D97" t="s">
@@ -5641,7 +5650,7 @@
       <c r="B98" t="s">
         <v>150</v>
       </c>
-      <c r="C98" t="s">
+      <c r="C98" s="7" t="s">
         <v>201</v>
       </c>
       <c r="D98" t="s">
@@ -5688,7 +5697,7 @@
       <c r="B99" t="s">
         <v>154</v>
       </c>
-      <c r="C99" t="s">
+      <c r="C99" s="7" t="s">
         <v>201</v>
       </c>
       <c r="D99" t="s">
@@ -5735,7 +5744,7 @@
       <c r="B100" t="s">
         <v>155</v>
       </c>
-      <c r="C100" t="s">
+      <c r="C100" s="7" t="s">
         <v>201</v>
       </c>
       <c r="D100" t="s">
@@ -5782,7 +5791,7 @@
       <c r="B101" t="s">
         <v>149</v>
       </c>
-      <c r="C101" t="s">
+      <c r="C101" s="7" t="s">
         <v>184</v>
       </c>
       <c r="D101" t="s">
@@ -5829,7 +5838,7 @@
       <c r="B102" t="s">
         <v>146</v>
       </c>
-      <c r="C102" t="s">
+      <c r="C102" s="7" t="s">
         <v>202</v>
       </c>
       <c r="D102" t="s">
@@ -5876,7 +5885,7 @@
       <c r="B103" t="s">
         <v>148</v>
       </c>
-      <c r="C103" t="s">
+      <c r="C103" s="7" t="s">
         <v>202</v>
       </c>
       <c r="D103" t="s">
@@ -5923,7 +5932,7 @@
       <c r="B104" t="s">
         <v>141</v>
       </c>
-      <c r="C104" t="s">
+      <c r="C104" s="7" t="s">
         <v>203</v>
       </c>
       <c r="D104" t="s">
@@ -5970,7 +5979,7 @@
       <c r="B105" t="s">
         <v>138</v>
       </c>
-      <c r="C105" t="s">
+      <c r="C105" s="7" t="s">
         <v>204</v>
       </c>
       <c r="D105" t="s">
@@ -6017,7 +6026,7 @@
       <c r="B106" t="s">
         <v>139</v>
       </c>
-      <c r="C106" t="s">
+      <c r="C106" s="7" t="s">
         <v>204</v>
       </c>
       <c r="D106" t="s">
@@ -6064,7 +6073,7 @@
       <c r="B107" t="s">
         <v>136</v>
       </c>
-      <c r="C107" t="s">
+      <c r="C107" s="7" t="s">
         <v>204</v>
       </c>
       <c r="D107" t="s">
@@ -6111,7 +6120,7 @@
       <c r="B108" t="s">
         <v>143</v>
       </c>
-      <c r="C108" t="s">
+      <c r="C108" s="7" t="s">
         <v>202</v>
       </c>
       <c r="D108" t="s">
@@ -6158,7 +6167,7 @@
       <c r="B109" t="s">
         <v>170</v>
       </c>
-      <c r="C109" t="s">
+      <c r="C109" s="7" t="s">
         <v>205</v>
       </c>
       <c r="D109" t="s">
@@ -6205,7 +6214,7 @@
       <c r="B110" t="s">
         <v>171</v>
       </c>
-      <c r="C110" t="s">
+      <c r="C110" s="7" t="s">
         <v>205</v>
       </c>
       <c r="D110" t="s">
@@ -6252,7 +6261,7 @@
       <c r="B111" t="s">
         <v>172</v>
       </c>
-      <c r="C111" t="s">
+      <c r="C111" s="7" t="s">
         <v>205</v>
       </c>
       <c r="D111" t="s">
@@ -6299,7 +6308,7 @@
       <c r="B112" t="s">
         <v>149</v>
       </c>
-      <c r="C112" t="s">
+      <c r="C112" s="7" t="s">
         <v>206</v>
       </c>
       <c r="D112" t="s">
@@ -6346,7 +6355,7 @@
       <c r="B113" t="s">
         <v>149</v>
       </c>
-      <c r="C113" t="s">
+      <c r="C113" s="7" t="s">
         <v>207</v>
       </c>
       <c r="D113" t="s">
@@ -6393,7 +6402,7 @@
       <c r="B114" t="s">
         <v>155</v>
       </c>
-      <c r="C114" t="s">
+      <c r="C114" s="7" t="s">
         <v>207</v>
       </c>
       <c r="D114" t="s">
@@ -6440,7 +6449,7 @@
       <c r="B115" t="s">
         <v>173</v>
       </c>
-      <c r="C115" t="s">
+      <c r="C115" s="7" t="s">
         <v>186</v>
       </c>
       <c r="D115" t="s">
@@ -6487,7 +6496,7 @@
       <c r="B116" t="s">
         <v>174</v>
       </c>
-      <c r="C116" t="s">
+      <c r="C116" s="7" t="s">
         <v>187</v>
       </c>
       <c r="D116" t="s">
@@ -6534,7 +6543,7 @@
       <c r="B117" t="s">
         <v>175</v>
       </c>
-      <c r="C117" t="s">
+      <c r="C117" s="7" t="s">
         <v>187</v>
       </c>
       <c r="D117" t="s">
@@ -6581,7 +6590,7 @@
       <c r="B118" t="s">
         <v>176</v>
       </c>
-      <c r="C118" t="s">
+      <c r="C118" s="7" t="s">
         <v>187</v>
       </c>
       <c r="D118" t="s">
@@ -6628,7 +6637,7 @@
       <c r="B119" t="s">
         <v>177</v>
       </c>
-      <c r="C119" t="s">
+      <c r="C119" s="7" t="s">
         <v>187</v>
       </c>
       <c r="D119" t="s">
@@ -6675,7 +6684,7 @@
       <c r="B120" t="s">
         <v>178</v>
       </c>
-      <c r="C120" t="s">
+      <c r="C120" s="7" t="s">
         <v>187</v>
       </c>
       <c r="D120" t="s">

</xml_diff>

<commit_message>
Updated sensitivity analysis code, still need to add intercepts. Created new files for thorough datasheet proofreading
</commit_message>
<xml_diff>
--- a/data/cyano_atx_24.xlsx
+++ b/data/cyano_atx_24.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jld/Documents/Github/River_HAB_Modeling/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B2199ED-7C15-C945-B470-AED90827D9E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB3631FF-D213-F44A-87C6-734065D07D88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="800" yWindow="760" windowWidth="27700" windowHeight="18040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1274" uniqueCount="219">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1273" uniqueCount="219">
   <si>
     <t>ESF</t>
   </si>
@@ -790,7 +790,7 @@
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -2677,28 +2677,28 @@
     </row>
     <row r="33" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B33" t="s">
-        <v>149</v>
+        <v>158</v>
       </c>
       <c r="C33" s="7" t="s">
         <v>187</v>
       </c>
       <c r="D33" s="9" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="E33">
-        <v>0.47499999999999998</v>
+        <v>2.4969999999999999</v>
       </c>
       <c r="F33">
-        <v>0.159</v>
+        <v>0.17</v>
       </c>
       <c r="G33" t="s">
         <v>208</v>
       </c>
       <c r="H33">
-        <v>9.0999999999999998E-2</v>
+        <v>9.7000000000000003E-2</v>
       </c>
       <c r="I33" t="s">
         <v>208</v>
@@ -2707,10 +2707,10 @@
         <v>0.05</v>
       </c>
       <c r="K33">
-        <v>0.43</v>
+        <v>1.901</v>
       </c>
       <c r="L33">
-        <v>4.4999999999999998E-2</v>
+        <v>0.59599999999999997</v>
       </c>
       <c r="M33" t="s">
         <v>208</v>
@@ -2719,17 +2719,17 @@
         <v>208</v>
       </c>
       <c r="O33">
-        <v>0.47499999999999998</v>
+        <v>2.4969999999999999</v>
       </c>
       <c r="Q33" s="9"/>
       <c r="R33" s="9"/>
     </row>
     <row r="34" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B34" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="C34" s="7" t="s">
         <v>187</v>
@@ -2738,28 +2738,28 @@
         <v>218</v>
       </c>
       <c r="E34">
-        <v>0.47099999999999997</v>
+        <v>0.47499999999999998</v>
       </c>
       <c r="F34">
-        <v>0.214</v>
+        <v>0.159</v>
       </c>
       <c r="G34" t="s">
         <v>208</v>
       </c>
       <c r="H34">
-        <v>0.122</v>
+        <v>9.0999999999999998E-2</v>
       </c>
       <c r="I34" t="s">
         <v>208</v>
       </c>
       <c r="J34">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="K34">
-        <v>0.41799999999999998</v>
+        <v>0.43</v>
       </c>
       <c r="L34">
-        <v>5.2999999999999999E-2</v>
+        <v>4.4999999999999998E-2</v>
       </c>
       <c r="M34" t="s">
         <v>208</v>
@@ -2768,17 +2768,17 @@
         <v>208</v>
       </c>
       <c r="O34">
-        <v>0.47099999999999997</v>
+        <v>0.47499999999999998</v>
       </c>
       <c r="Q34" s="9"/>
       <c r="R34" s="9"/>
     </row>
     <row r="35" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B35" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C35" s="7" t="s">
         <v>187</v>
@@ -2787,28 +2787,28 @@
         <v>218</v>
       </c>
       <c r="E35">
-        <v>0.66800000000000004</v>
+        <v>0.47099999999999997</v>
       </c>
       <c r="F35">
-        <v>0.17299999999999999</v>
+        <v>0.214</v>
       </c>
       <c r="G35" t="s">
         <v>208</v>
       </c>
       <c r="H35">
-        <v>9.9000000000000005E-2</v>
+        <v>0.122</v>
       </c>
       <c r="I35" t="s">
         <v>208</v>
       </c>
       <c r="J35">
-        <v>0.05</v>
+        <v>0.06</v>
       </c>
       <c r="K35">
-        <v>0.497</v>
+        <v>0.41799999999999998</v>
       </c>
       <c r="L35">
-        <v>0.17100000000000001</v>
+        <v>5.2999999999999999E-2</v>
       </c>
       <c r="M35" t="s">
         <v>208</v>
@@ -2817,35 +2817,35 @@
         <v>208</v>
       </c>
       <c r="O35">
-        <v>0.66800000000000004</v>
+        <v>0.47099999999999997</v>
       </c>
       <c r="Q35" s="9"/>
       <c r="R35" s="9"/>
     </row>
     <row r="36" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B36" t="s">
-        <v>149</v>
+        <v>157</v>
       </c>
       <c r="C36" s="7" t="s">
         <v>187</v>
       </c>
       <c r="D36" s="9" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="E36">
-        <v>2.4969999999999999</v>
+        <v>0.66800000000000004</v>
       </c>
       <c r="F36">
-        <v>0.17</v>
+        <v>0.17299999999999999</v>
       </c>
       <c r="G36" t="s">
         <v>208</v>
       </c>
       <c r="H36">
-        <v>9.7000000000000003E-2</v>
+        <v>9.9000000000000005E-2</v>
       </c>
       <c r="I36" t="s">
         <v>208</v>
@@ -2854,10 +2854,10 @@
         <v>0.05</v>
       </c>
       <c r="K36">
-        <v>1.901</v>
+        <v>0.497</v>
       </c>
       <c r="L36">
-        <v>0.59599999999999997</v>
+        <v>0.17100000000000001</v>
       </c>
       <c r="M36" t="s">
         <v>208</v>
@@ -2866,7 +2866,7 @@
         <v>208</v>
       </c>
       <c r="O36">
-        <v>2.4969999999999999</v>
+        <v>0.66800000000000004</v>
       </c>
       <c r="Q36" s="9"/>
       <c r="R36" s="9"/>
@@ -5903,8 +5903,8 @@
       <c r="N98" t="s">
         <v>208</v>
       </c>
-      <c r="O98" t="s">
-        <v>208</v>
+      <c r="O98">
+        <v>8.7999999999999995E-2</v>
       </c>
       <c r="Q98" s="9"/>
       <c r="R98" s="9"/>

</xml_diff>